<commit_message>
PO2026066: assign B/L vs PL weight difference to empty cartons
The 145 empty printed cartons (48191000) have no weight on the packing list.
The B/L minus PL difference (274.21 kg, 3.19 m3, ~1.89 kg/box) is assigned
to them, so totals now match the B/L (15,690.00 kg). Marked as derived and
to be confirmed with the shipper.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V7ceSf8byPvxCS9kda91VB
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_ALL2COVER_PO2026066.xlsx
+++ b/output/HS_Code_Summary_ALL2COVER_PO2026066.xlsx
@@ -966,12 +966,18 @@
       <c r="E9" s="4" t="n">
         <v>145</v>
       </c>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
+      <c r="F9" s="6" t="n">
+        <v>274.21</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>274.21</v>
+      </c>
       <c r="H9" s="5" t="n">
         <v>217.5</v>
       </c>
-      <c r="I9" s="4" t="n"/>
+      <c r="I9" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
           <t>48</t>
@@ -989,7 +995,7 @@
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>Hmotnost CHYBÍ – na packing listu není u krabic uvedena (nutno doplnit od odesílatele).</t>
+          <t>⚠️ Hmotnost ODVOZENA (na PL chybí): rozdíl B/L 15 690,00 kg − PL 15 415,79 kg = 274,21 kg (≈1,89 kg/krabice; objem 60,80 − 57,61 = 3,19 m³). Čistá = hrubá (zboží = samotné krabice). Potvrdit u odesílatele.</t>
         </is>
       </c>
     </row>
@@ -1059,10 +1065,10 @@
         <v>558175</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>14281.79</v>
+        <v>14556</v>
       </c>
       <c r="G11" s="11" t="n">
-        <v>15415.79</v>
+        <v>15690</v>
       </c>
       <c r="H11" s="11" t="n">
         <v>58528.65</v>
@@ -1143,7 +1149,7 @@
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>Čistá / hrubá dle PL: 14 281,79 / 15 415,79 kg, 1134 ctn, 57,61 m³. ⚠️ B/L uvádí 15 690,00 kg a 60,80 m³ (rozdíl +274,21 kg). Krabice (48191000) bez hmotnosti.</t>
+          <t>Čistá / hrubá dle PL: 14 281,79 / 15 415,79 kg, 1134 ctn, 57,61 m³; B/L: 15 690,00 kg, 60,80 m³. ⚠️ Rozdíl 274,21 kg / 3,19 m³ přiřazen krabicím 48191000 (145 ks, na PL bez hmotnosti; mimo 1134 ctn) → součty sedí na B/L (15 690,00 kg). Odvozeno – potvrdit u odesílatele.</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1303,6 +1309,11 @@
           <t>m³</t>
         </is>
       </c>
+      <c r="L1" s="15" t="inlineStr">
+        <is>
+          <t>Poznámka</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -3254,6 +3265,23 @@
       </c>
       <c r="G49" t="n">
         <v>217.5</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" t="n">
+        <v>274.21</v>
+      </c>
+      <c r="J49" t="n">
+        <v>274.21</v>
+      </c>
+      <c r="K49" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Hmotnost/objem odvozeny z rozdílu B/L − PL (na PL chybí)</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>